<commit_message>
chore: establish public repository governance
</commit_message>
<xml_diff>
--- a/tests/support/fixtures/spreadsheet/color-filtered-roster.xlsx
+++ b/tests/support/fixtures/spreadsheet/color-filtered-roster.xlsx
@@ -536,7 +536,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="10003182" scaled="1"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -555,7 +555,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="10003182" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>

</xml_diff>